<commit_message>
Replace deprecated use_container_width=True with width="stretch".  Add 2026Q2 results for AAL and LUV.
</commit_message>
<xml_diff>
--- a/airline-dashboard/data/manual/airline_financial_data.xlsx
+++ b/airline-dashboard/data/manual/airline_financial_data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trica\OneDrive\Documents\School\UNCC\Personal Projects\US Airlines Financials Project\airline_financials\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0f26b992e1a44723/Documents/GitHub Repos/airline_financials/airline-dashboard/data/manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{826EDDCB-8DC5-48D4-92ED-2287CEBE3206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{826EDDCB-8DC5-48D4-92ED-2287CEBE3206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{504DDDFE-45E9-48EE-AC9F-46D174CB1856}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5CC2E0DD-0C2A-471D-BE08-E27D8B31800B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5CC2E0DD-0C2A-471D-BE08-E27D8B31800B}"/>
   </bookViews>
   <sheets>
     <sheet name="airline_financials" sheetId="2" r:id="rId1"/>
@@ -957,22 +957,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95BF35CD-6CF2-4D2E-9294-3A1A732D8FBE}">
   <dimension ref="A1:K209"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="5.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.6640625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="16.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="9" width="17.109375" customWidth="1"/>
-    <col min="10" max="10" width="13.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="5.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="17.140625" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="11.7109375" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1007,7 +1007,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2018</v>
       </c>
@@ -1042,7 +1042,7 @@
         <v>29000000</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2018</v>
       </c>
@@ -1074,7 +1074,7 @@
         <v>188000000</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2018</v>
       </c>
@@ -1106,7 +1106,7 @@
         <v>17000000</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2018</v>
       </c>
@@ -1141,7 +1141,7 @@
         <v>63000000</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2018</v>
       </c>
@@ -1176,7 +1176,7 @@
         <v>404000000</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2018</v>
       </c>
@@ -1208,7 +1208,7 @@
         <v>108000000</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2018</v>
       </c>
@@ -1243,7 +1243,7 @@
         <v>43000000</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2018</v>
       </c>
@@ -1278,7 +1278,7 @@
         <v>399000000</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2018</v>
       </c>
@@ -1310,7 +1310,7 @@
         <v>127000000</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2018</v>
       </c>
@@ -1345,7 +1345,7 @@
         <v>40000000</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2018</v>
       </c>
@@ -1380,7 +1380,7 @@
         <v>311000000</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2018</v>
       </c>
@@ -1415,7 +1415,7 @@
         <v>82000000</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2018</v>
       </c>
@@ -1450,7 +1450,7 @@
         <v>175000000</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2018</v>
       </c>
@@ -1485,7 +1485,7 @@
         <v>1301000000</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2018</v>
       </c>
@@ -1520,7 +1520,7 @@
         <v>334000000</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2019</v>
       </c>
@@ -1555,7 +1555,7 @@
         <v>20000000</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2019</v>
       </c>
@@ -1590,7 +1590,7 @@
         <v>220000000</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2019</v>
       </c>
@@ -1622,7 +1622,7 @@
         <v>33000000</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2019</v>
       </c>
@@ -1657,7 +1657,7 @@
         <v>67000000</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2019</v>
       </c>
@@ -1692,7 +1692,7 @@
         <v>518000000</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2019</v>
       </c>
@@ -1724,7 +1724,7 @@
         <v>161000000</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2019</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>52000000</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2019</v>
       </c>
@@ -1794,7 +1794,7 @@
         <v>517000000</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2019</v>
       </c>
@@ -1826,7 +1826,7 @@
         <v>174000000</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>2019</v>
       </c>
@@ -1861,7 +1861,7 @@
         <v>74000000</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>2019</v>
       </c>
@@ -1896,7 +1896,7 @@
         <v>387000000</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>2019</v>
       </c>
@@ -1931,7 +1931,7 @@
         <v>123000000</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>2019</v>
       </c>
@@ -1966,7 +1966,7 @@
         <v>213000000</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>2019</v>
       </c>
@@ -2001,7 +2001,7 @@
         <v>1643000000</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>2019</v>
       </c>
@@ -2036,7 +2036,7 @@
         <v>491000000</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>2020</v>
       </c>
@@ -2071,7 +2071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>2020</v>
       </c>
@@ -2106,7 +2106,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>2020</v>
       </c>
@@ -2138,7 +2138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>2020</v>
       </c>
@@ -2173,7 +2173,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>2020</v>
       </c>
@@ -2208,7 +2208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>2020</v>
       </c>
@@ -2240,7 +2240,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>2020</v>
       </c>
@@ -2275,7 +2275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>2020</v>
       </c>
@@ -2310,7 +2310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>2020</v>
       </c>
@@ -2342,7 +2342,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>2020</v>
       </c>
@@ -2377,7 +2377,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>2020</v>
       </c>
@@ -2412,7 +2412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>2020</v>
       </c>
@@ -2447,7 +2447,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>2020</v>
       </c>
@@ -2482,7 +2482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>2020</v>
       </c>
@@ -2517,7 +2517,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>2020</v>
       </c>
@@ -2552,7 +2552,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>2021</v>
       </c>
@@ -2587,7 +2587,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>2021</v>
       </c>
@@ -2622,7 +2622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>2021</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>2021</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>2021</v>
       </c>
@@ -2724,7 +2724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>2021</v>
       </c>
@@ -2756,7 +2756,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>2021</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>2021</v>
       </c>
@@ -2826,7 +2826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>2021</v>
       </c>
@@ -2858,7 +2858,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>2021</v>
       </c>
@@ -2893,7 +2893,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>2021</v>
       </c>
@@ -2928,7 +2928,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>2021</v>
       </c>
@@ -2963,7 +2963,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>2021</v>
       </c>
@@ -2998,7 +2998,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>2021</v>
       </c>
@@ -3033,7 +3033,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>2021</v>
       </c>
@@ -3068,7 +3068,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>2022</v>
       </c>
@@ -3103,7 +3103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>2022</v>
       </c>
@@ -3138,7 +3138,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>2022</v>
       </c>
@@ -3170,7 +3170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>2022</v>
       </c>
@@ -3205,7 +3205,7 @@
         <v>64000000</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>2022</v>
       </c>
@@ -3240,7 +3240,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>2022</v>
       </c>
@@ -3272,7 +3272,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>2022</v>
       </c>
@@ -3307,7 +3307,7 @@
         <v>59000000</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>2022</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>237000000</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>2022</v>
       </c>
@@ -3374,7 +3374,7 @@
         <v>8000000</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>2022</v>
       </c>
@@ -3409,7 +3409,7 @@
         <v>88000000</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>2022</v>
       </c>
@@ -3444,7 +3444,7 @@
         <v>272000000</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>2022</v>
       </c>
@@ -3479,7 +3479,7 @@
         <v>125000000</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>2022</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>211000000</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>2022</v>
       </c>
@@ -3549,7 +3549,7 @@
         <v>563000000</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>2022</v>
       </c>
@@ -3584,7 +3584,7 @@
         <v>133000000</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>2023</v>
       </c>
@@ -3619,7 +3619,7 @@
         <v>35000000</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>2023</v>
       </c>
@@ -3654,7 +3654,7 @@
         <v>72000000</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>2023</v>
       </c>
@@ -3686,7 +3686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>2023</v>
       </c>
@@ -3721,7 +3721,7 @@
         <v>173000000</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>2023</v>
       </c>
@@ -3756,7 +3756,7 @@
         <v>595000000</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>2023</v>
       </c>
@@ -3788,7 +3788,7 @@
         <v>220000000</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>2023</v>
       </c>
@@ -3823,7 +3823,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>2023</v>
       </c>
@@ -3858,7 +3858,7 @@
         <v>417000000</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>2023</v>
       </c>
@@ -3890,7 +3890,7 @@
         <v>301000000</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>2023</v>
       </c>
@@ -3925,7 +3925,7 @@
         <v>53000000</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>2023</v>
       </c>
@@ -3960,7 +3960,7 @@
         <v>299000000</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>2023</v>
       </c>
@@ -3995,7 +3995,7 @@
         <v>160000000</v>
       </c>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>2023</v>
       </c>
@@ -4030,7 +4030,7 @@
         <v>261000000</v>
       </c>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>2023</v>
       </c>
@@ -4065,7 +4065,7 @@
         <v>1383000000</v>
       </c>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>2023</v>
       </c>
@@ -4100,7 +4100,7 @@
         <v>681000000</v>
       </c>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>2024</v>
       </c>
@@ -4136,7 +4136,7 @@
         <v>610559</v>
       </c>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>2024</v>
       </c>
@@ -4171,7 +4171,7 @@
         <v>125000000</v>
       </c>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>2024</v>
       </c>
@@ -4203,7 +4203,7 @@
         <v>3000000</v>
       </c>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>2024</v>
       </c>
@@ -4239,7 +4239,7 @@
         <v>120716144</v>
       </c>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>2024</v>
       </c>
@@ -4274,7 +4274,7 @@
         <v>519000000</v>
       </c>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>2024</v>
       </c>
@@ -4306,7 +4306,7 @@
         <v>185000000</v>
       </c>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>2024</v>
       </c>
@@ -4342,7 +4342,7 @@
         <v>7762816</v>
       </c>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>2024</v>
       </c>
@@ -4377,7 +4377,7 @@
         <v>320000000</v>
       </c>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>2024</v>
       </c>
@@ -4409,7 +4409,7 @@
         <v>231000000</v>
       </c>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>2017</v>
       </c>
@@ -4444,7 +4444,7 @@
         <v>241000000</v>
       </c>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>2016</v>
       </c>
@@ -4479,7 +4479,7 @@
         <v>314000000</v>
       </c>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>2015</v>
       </c>
@@ -4514,7 +4514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>2014</v>
       </c>
@@ -4549,7 +4549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>2017</v>
       </c>
@@ -4584,7 +4584,7 @@
         <v>1065000000</v>
       </c>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>2016</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>1115000000</v>
       </c>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A107">
         <v>2015</v>
       </c>
@@ -4654,7 +4654,7 @@
         <v>1490000000</v>
       </c>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A108">
         <v>2014</v>
       </c>
@@ -4689,7 +4689,7 @@
         <v>1085000000</v>
       </c>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A109">
         <v>2017</v>
       </c>
@@ -4724,7 +4724,7 @@
         <v>349000000</v>
       </c>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A110">
         <v>2016</v>
       </c>
@@ -4759,7 +4759,7 @@
         <v>628000000</v>
       </c>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A111">
         <v>2015</v>
       </c>
@@ -4794,7 +4794,7 @@
         <v>698000000</v>
       </c>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A112">
         <v>2014</v>
       </c>
@@ -4829,7 +4829,7 @@
         <v>235000000</v>
       </c>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A113">
         <v>2023</v>
       </c>
@@ -4864,7 +4864,7 @@
         <v>110000000</v>
       </c>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A114">
         <v>2022</v>
       </c>
@@ -4899,7 +4899,7 @@
         <v>127000000</v>
       </c>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A115">
         <v>2021</v>
       </c>
@@ -4934,7 +4934,7 @@
         <v>230000000</v>
       </c>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A116">
         <v>2020</v>
       </c>
@@ -4969,7 +4969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A117">
         <v>2019</v>
       </c>
@@ -5004,7 +5004,7 @@
         <v>695000000</v>
       </c>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A118">
         <v>2018</v>
       </c>
@@ -5039,7 +5039,7 @@
         <v>580000000</v>
       </c>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A119">
         <v>2017</v>
       </c>
@@ -5074,7 +5074,7 @@
         <v>579000000</v>
       </c>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A120">
         <v>2016</v>
       </c>
@@ -5109,7 +5109,7 @@
         <v>645000000</v>
       </c>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A121">
         <v>2015</v>
       </c>
@@ -5144,7 +5144,7 @@
         <v>655000000</v>
       </c>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A122">
         <v>2014</v>
       </c>
@@ -5179,7 +5179,7 @@
         <v>374000000</v>
       </c>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A123">
         <v>2024</v>
       </c>
@@ -5214,7 +5214,7 @@
         <v>18000000</v>
       </c>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A124">
         <v>2024</v>
       </c>
@@ -5249,7 +5249,7 @@
         <v>31000000</v>
       </c>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A125">
         <v>2024</v>
       </c>
@@ -5284,7 +5284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A126">
         <v>2017</v>
       </c>
@@ -5319,7 +5319,7 @@
         <v>31000000</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A127">
         <v>2017</v>
       </c>
@@ -5354,7 +5354,7 @@
         <v>94000000</v>
       </c>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A128">
         <v>2017</v>
       </c>
@@ -5389,7 +5389,7 @@
         <v>70000000</v>
       </c>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A129">
         <v>2017</v>
       </c>
@@ -5424,7 +5424,7 @@
         <v>47000000</v>
       </c>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A130">
         <v>2016</v>
       </c>
@@ -5459,7 +5459,7 @@
         <v>73000000</v>
       </c>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A131">
         <v>2016</v>
       </c>
@@ -5494,7 +5494,7 @@
         <v>98000000</v>
       </c>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A132">
         <v>2016</v>
       </c>
@@ -5529,7 +5529,7 @@
         <v>86000000</v>
       </c>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A133">
         <v>2016</v>
       </c>
@@ -5564,7 +5564,7 @@
         <v>57000000</v>
       </c>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A134">
         <v>2015</v>
       </c>
@@ -5599,7 +5599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A135">
         <v>2015</v>
       </c>
@@ -5634,7 +5634,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A136">
         <v>2015</v>
       </c>
@@ -5669,7 +5669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A137">
         <v>2015</v>
       </c>
@@ -5704,7 +5704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A138">
         <v>2014</v>
       </c>
@@ -5739,7 +5739,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A139">
         <v>2014</v>
       </c>
@@ -5774,7 +5774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A140">
         <v>2014</v>
       </c>
@@ -5809,7 +5809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A141">
         <v>2014</v>
       </c>
@@ -5844,7 +5844,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A142">
         <v>2017</v>
       </c>
@@ -5876,7 +5876,7 @@
         <v>151000000</v>
       </c>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A143">
         <v>2017</v>
       </c>
@@ -5908,7 +5908,7 @@
         <v>338000000</v>
       </c>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A144">
         <v>2017</v>
       </c>
@@ -5940,7 +5940,7 @@
         <v>314000000</v>
       </c>
     </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A145">
         <v>2017</v>
       </c>
@@ -5975,7 +5975,7 @@
         <v>262000000</v>
       </c>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A146">
         <v>2016</v>
       </c>
@@ -6007,7 +6007,7 @@
         <v>272000000</v>
       </c>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A147">
         <v>2016</v>
       </c>
@@ -6039,7 +6039,7 @@
         <v>324000000</v>
       </c>
     </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A148">
         <v>2016</v>
       </c>
@@ -6071,7 +6071,7 @@
         <v>326000000</v>
       </c>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A149">
         <v>2016</v>
       </c>
@@ -6106,7 +6106,7 @@
         <v>193000000</v>
       </c>
     </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A150">
         <v>2015</v>
       </c>
@@ -6138,7 +6138,7 @@
         <v>136000000</v>
       </c>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A151">
         <v>2015</v>
       </c>
@@ -6170,7 +6170,7 @@
         <v>411000000</v>
       </c>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A152">
         <v>2015</v>
       </c>
@@ -6202,7 +6202,7 @@
         <v>563000000</v>
       </c>
     </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A153">
         <v>2015</v>
       </c>
@@ -6237,7 +6237,7 @@
         <v>380000000</v>
       </c>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A154">
         <v>2014</v>
       </c>
@@ -6269,7 +6269,7 @@
         <v>99000000</v>
       </c>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A155">
         <v>2014</v>
       </c>
@@ -6301,7 +6301,7 @@
         <v>340000000</v>
       </c>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A156">
         <v>2014</v>
       </c>
@@ -6333,7 +6333,7 @@
         <v>384000000</v>
       </c>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A157">
         <v>2014</v>
       </c>
@@ -6368,7 +6368,7 @@
         <v>262000000</v>
       </c>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A158">
         <v>2017</v>
       </c>
@@ -6400,7 +6400,7 @@
         <v>28000000</v>
       </c>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A159">
         <v>2017</v>
       </c>
@@ -6432,7 +6432,7 @@
         <v>140000000</v>
       </c>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A160">
         <v>2017</v>
       </c>
@@ -6464,7 +6464,7 @@
         <v>109000000</v>
       </c>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A161">
         <v>2017</v>
       </c>
@@ -6499,7 +6499,7 @@
         <v>73000000</v>
       </c>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A162">
         <v>2016</v>
       </c>
@@ -6531,7 +6531,7 @@
         <v>94000000</v>
       </c>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A163">
         <v>2016</v>
       </c>
@@ -6563,7 +6563,7 @@
         <v>153000000</v>
       </c>
     </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A164">
         <v>2016</v>
       </c>
@@ -6595,7 +6595,7 @@
         <v>235000000</v>
       </c>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A165">
         <v>2016</v>
       </c>
@@ -6630,7 +6630,7 @@
         <v>145000000</v>
       </c>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A166">
         <v>2015</v>
       </c>
@@ -6662,7 +6662,7 @@
         <v>100000000</v>
       </c>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A167">
         <v>2015</v>
       </c>
@@ -6694,7 +6694,7 @@
         <v>195000000</v>
       </c>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A168">
         <v>2015</v>
       </c>
@@ -6726,7 +6726,7 @@
         <v>257000000</v>
       </c>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A169">
         <v>2015</v>
       </c>
@@ -6761,7 +6761,7 @@
         <v>146000000</v>
       </c>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A170">
         <v>2014</v>
       </c>
@@ -6793,7 +6793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A171">
         <v>2014</v>
       </c>
@@ -6825,7 +6825,7 @@
         <v>78000000</v>
       </c>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A172">
         <v>2014</v>
       </c>
@@ -6857,7 +6857,7 @@
         <v>103000000</v>
       </c>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A173">
         <v>2014</v>
       </c>
@@ -6892,7 +6892,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A174">
         <v>2024</v>
       </c>
@@ -6927,7 +6927,7 @@
         <v>425000000</v>
       </c>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A175">
         <v>2024</v>
       </c>
@@ -6962,7 +6962,7 @@
         <v>1389000000</v>
       </c>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A176">
         <v>2024</v>
       </c>
@@ -6997,7 +6997,7 @@
         <v>294000000</v>
       </c>
     </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A177">
         <v>2024</v>
       </c>
@@ -7032,7 +7032,7 @@
         <v>713000000</v>
       </c>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A178">
         <v>2024</v>
       </c>
@@ -7068,7 +7068,7 @@
         <v>98910482</v>
       </c>
     </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A179">
         <v>2024</v>
       </c>
@@ -7103,7 +7103,7 @@
         <v>228000000</v>
       </c>
     </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A180">
         <v>2024</v>
       </c>
@@ -7138,7 +7138,7 @@
         <v>54000000</v>
       </c>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A181">
         <v>2024</v>
       </c>
@@ -7173,7 +7173,7 @@
         <v>103000000</v>
       </c>
     </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A182">
         <v>2025</v>
       </c>
@@ -7208,7 +7208,7 @@
         <v>124000000</v>
       </c>
     </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A183">
         <v>2025</v>
       </c>
@@ -7240,7 +7240,7 @@
         <v>43000000</v>
       </c>
     </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A184">
         <v>2025</v>
       </c>
@@ -7275,7 +7275,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A185">
         <v>2025</v>
       </c>
@@ -7310,7 +7310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A186">
         <v>2025</v>
       </c>
@@ -7345,7 +7345,7 @@
         <v>470000000</v>
       </c>
     </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A187">
         <v>2025</v>
       </c>
@@ -7377,7 +7377,7 @@
         <v>188000000</v>
       </c>
     </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A188">
         <v>2025</v>
       </c>
@@ -7409,11 +7409,10 @@
         <v>24217000000</v>
       </c>
       <c r="K188">
-        <f>ROUND($K$201*(((D188-F188)/($D$201-$F$201))/(((D200-F200)/($D$201-$F$201))+((D188-F188)/($D$201-$F$201)))),0)</f>
-        <v>39360025</v>
-      </c>
-    </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.3">
+        <v>41000000</v>
+      </c>
+    </row>
+    <row r="189" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A189">
         <v>2025</v>
       </c>
@@ -7448,7 +7447,7 @@
         <v>14000000</v>
       </c>
     </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A190">
         <v>2025</v>
       </c>
@@ -7483,7 +7482,7 @@
         <v>392000000</v>
       </c>
     </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A191">
         <v>2025</v>
       </c>
@@ -7515,7 +7514,7 @@
         <v>228000000</v>
       </c>
     </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A192">
         <v>2025</v>
       </c>
@@ -7550,7 +7549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A193">
         <v>2025</v>
       </c>
@@ -7585,7 +7584,7 @@
         <v>11000000</v>
       </c>
     </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A194">
         <v>2025</v>
       </c>
@@ -7620,7 +7619,7 @@
         <v>351000000</v>
       </c>
     </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A195">
         <v>2025</v>
       </c>
@@ -7655,7 +7654,7 @@
         <v>1337000000</v>
       </c>
     </row>
-    <row r="196" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A196">
         <v>2025</v>
       </c>
@@ -7690,7 +7689,7 @@
         <v>244000000</v>
       </c>
     </row>
-    <row r="197" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A197">
         <v>2025</v>
       </c>
@@ -7725,7 +7724,7 @@
         <v>704000000</v>
       </c>
     </row>
-    <row r="198" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A198">
         <v>2025</v>
       </c>
@@ -7760,7 +7759,7 @@
         <v>71000000</v>
       </c>
     </row>
-    <row r="199" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A199">
         <v>2025</v>
       </c>
@@ -7795,7 +7794,7 @@
         <v>97000000</v>
       </c>
     </row>
-    <row r="200" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A200">
         <v>2025</v>
       </c>
@@ -7831,7 +7830,7 @@
         <v>15639975</v>
       </c>
     </row>
-    <row r="201" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A201">
         <v>2025</v>
       </c>
@@ -7866,7 +7865,7 @@
         <v>55000000</v>
       </c>
     </row>
-    <row r="202" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A202">
         <v>2026</v>
       </c>
@@ -7901,7 +7900,7 @@
         <v>165000000</v>
       </c>
     </row>
-    <row r="203" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A203">
         <v>2026</v>
       </c>
@@ -7933,7 +7932,7 @@
         <v>59000000</v>
       </c>
     </row>
-    <row r="204" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A204">
         <v>2026</v>
       </c>
@@ -7968,7 +7967,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="205" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A205">
         <v>2026</v>
       </c>
@@ -8003,7 +8002,7 @@
         <v>50000000</v>
       </c>
     </row>
-    <row r="206" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A206">
         <v>2026</v>
       </c>
@@ -8038,7 +8037,7 @@
         <v>328000000</v>
       </c>
     </row>
-    <row r="207" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A207">
         <v>2026</v>
       </c>
@@ -8070,7 +8069,7 @@
         <v>90000000</v>
       </c>
     </row>
-    <row r="208" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A208">
         <v>2026</v>
       </c>
@@ -8080,8 +8079,29 @@
       <c r="C208" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="209" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="D208">
+        <v>16735000000</v>
+      </c>
+      <c r="E208">
+        <v>15214000000</v>
+      </c>
+      <c r="F208">
+        <v>16289000000</v>
+      </c>
+      <c r="G208">
+        <v>71000000</v>
+      </c>
+      <c r="H208">
+        <v>68118000000</v>
+      </c>
+      <c r="I208">
+        <v>81843000000</v>
+      </c>
+      <c r="K208">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="209" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A209">
         <v>2026</v>
       </c>
@@ -8090,6 +8110,27 @@
       </c>
       <c r="C209" t="s">
         <v>13</v>
+      </c>
+      <c r="D209">
+        <v>8432000000</v>
+      </c>
+      <c r="E209">
+        <v>7745000000</v>
+      </c>
+      <c r="F209">
+        <v>8147000000</v>
+      </c>
+      <c r="G209">
+        <v>285000000</v>
+      </c>
+      <c r="H209">
+        <v>37346000000</v>
+      </c>
+      <c r="I209">
+        <v>47093000000</v>
+      </c>
+      <c r="K209">
+        <v>53000000</v>
       </c>
     </row>
   </sheetData>
@@ -8100,13 +8141,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{47E8CB36-28FD-4A01-8E6F-FAD97027E6F9}">
   <dimension ref="A1:E25"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8123,7 +8164,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2013</v>
       </c>
@@ -8140,7 +8181,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2014</v>
       </c>
@@ -8157,7 +8198,7 @@
         <v>1000000000</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2015</v>
       </c>
@@ -8174,7 +8215,7 @@
         <v>3600000000</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2016</v>
       </c>
@@ -8191,7 +8232,7 @@
         <v>4400000000</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2017</v>
       </c>
@@ -8208,7 +8249,7 @@
         <v>1600000000</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2018</v>
       </c>
@@ -8225,7 +8266,7 @@
         <v>800000000</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>2019</v>
       </c>
@@ -8242,7 +8283,7 @@
         <v>1100000000</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>2020</v>
       </c>
@@ -8259,7 +8300,7 @@
         <v>145000000</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>2013</v>
       </c>
@@ -8276,7 +8317,7 @@
         <v>250000000</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>2014</v>
       </c>
@@ -8293,7 +8334,7 @@
         <v>1100000000</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>2015</v>
       </c>
@@ -8310,7 +8351,7 @@
         <v>2200000000</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>2016</v>
       </c>
@@ -8327,7 +8368,7 @@
         <v>2600000000</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>2017</v>
       </c>
@@ -8344,7 +8385,7 @@
         <v>1700000000</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>2018</v>
       </c>
@@ -8361,7 +8402,7 @@
         <v>1600000000</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>2019</v>
       </c>
@@ -8378,7 +8419,7 @@
         <v>2000000000</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>2020</v>
       </c>
@@ -8395,7 +8436,7 @@
         <v>377620000</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>2013</v>
       </c>
@@ -8412,7 +8453,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>2014</v>
       </c>
@@ -8429,7 +8470,7 @@
         <v>320000000</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>2015</v>
       </c>
@@ -8446,7 +8487,7 @@
         <v>1200000000</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>2016</v>
       </c>
@@ -8463,7 +8504,7 @@
         <v>2600000000</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>2017</v>
       </c>
@@ -8480,7 +8521,7 @@
         <v>1800000000</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>2018</v>
       </c>
@@ -8497,7 +8538,7 @@
         <v>1200000000</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>2019</v>
       </c>
@@ -8514,7 +8555,7 @@
         <v>1600000000</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>2020</v>
       </c>
@@ -8539,16 +8580,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{490D347E-B079-4188-B046-54C6AF8BB324}">
   <dimension ref="A1:E7"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="4.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="7.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.88671875" style="1" customWidth="1"/>
+    <col min="1" max="1" width="4.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.85546875" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -8565,7 +8606,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>2020</v>
       </c>
@@ -8582,7 +8623,7 @@
         <v>1901355562.5899999</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2021</v>
       </c>
@@ -8599,7 +8640,7 @@
         <v>1082205377.28</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>2020</v>
       </c>
@@ -8616,7 +8657,7 @@
         <v>158535000</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>2021</v>
       </c>
@@ -8633,7 +8674,7 @@
         <v>83433000</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>2020</v>
       </c>
@@ -8650,7 +8691,7 @@
         <v>2293578491.5</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>2021</v>
       </c>

</xml_diff>

<commit_message>
Fill remaining passenger revenue gaps in 2018 manually by updating the manual data spreadsheet with ALK, JBLU, and HA data.
</commit_message>
<xml_diff>
--- a/airline-dashboard/data/manual/airline_financial_data.xlsx
+++ b/airline-dashboard/data/manual/airline_financial_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/0f26b992e1a44723/Documents/GitHub Repos/airline_financials/airline-dashboard/data/manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{826EDDCB-8DC5-48D4-92ED-2287CEBE3206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{623539DB-94CE-4819-82FE-06D2F853BFFB}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="13_ncr:1_{826EDDCB-8DC5-48D4-92ED-2287CEBE3206}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{129EAC36-BC35-44AC-9E23-3A745FA3494D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{5CC2E0DD-0C2A-471D-BE08-E27D8B31800B}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="23">
   <si>
     <t>Year</t>
   </si>
@@ -95,6 +95,15 @@
   </si>
   <si>
     <t>Operating Expenses</t>
+  </si>
+  <si>
+    <t>ALK</t>
+  </si>
+  <si>
+    <t>JBLU</t>
+  </si>
+  <si>
+    <t>HA</t>
   </si>
 </sst>
 </file>
@@ -639,10 +648,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -960,7 +965,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{95BF35CD-6CF2-4D2E-9294-3A1A732D8FBE}">
-  <dimension ref="A1:K249"/>
+  <dimension ref="A1:K264"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.5703125" bestFit="1" customWidth="1"/>
@@ -9055,6 +9060,216 @@
       </c>
       <c r="K249">
         <v>53000000</v>
+      </c>
+    </row>
+    <row r="250" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A250">
+        <v>2018</v>
+      </c>
+      <c r="B250">
+        <v>1</v>
+      </c>
+      <c r="C250" t="s">
+        <v>20</v>
+      </c>
+      <c r="E250">
+        <v>1684000000</v>
+      </c>
+    </row>
+    <row r="251" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A251">
+        <v>2018</v>
+      </c>
+      <c r="B251">
+        <v>2</v>
+      </c>
+      <c r="C251" t="s">
+        <v>20</v>
+      </c>
+      <c r="E251">
+        <v>1997000000</v>
+      </c>
+    </row>
+    <row r="252" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A252">
+        <v>2018</v>
+      </c>
+      <c r="B252">
+        <v>3</v>
+      </c>
+      <c r="C252" t="s">
+        <v>20</v>
+      </c>
+      <c r="E252">
+        <v>2043000000</v>
+      </c>
+    </row>
+    <row r="253" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A253">
+        <v>2018</v>
+      </c>
+      <c r="B253">
+        <v>4</v>
+      </c>
+      <c r="C253" t="s">
+        <v>20</v>
+      </c>
+      <c r="E253">
+        <v>1907000000</v>
+      </c>
+    </row>
+    <row r="254" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A254">
+        <v>2018</v>
+      </c>
+      <c r="B254" t="s">
+        <v>8</v>
+      </c>
+      <c r="C254" t="s">
+        <v>20</v>
+      </c>
+      <c r="E254">
+        <v>7631000000</v>
+      </c>
+    </row>
+    <row r="255" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A255">
+        <v>2018</v>
+      </c>
+      <c r="B255">
+        <v>1</v>
+      </c>
+      <c r="C255" t="s">
+        <v>21</v>
+      </c>
+      <c r="E255">
+        <v>1692000000</v>
+      </c>
+    </row>
+    <row r="256" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A256">
+        <v>2018</v>
+      </c>
+      <c r="B256">
+        <v>2</v>
+      </c>
+      <c r="C256" t="s">
+        <v>21</v>
+      </c>
+      <c r="E256">
+        <v>1858000000</v>
+      </c>
+    </row>
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A257">
+        <v>2018</v>
+      </c>
+      <c r="B257">
+        <v>3</v>
+      </c>
+      <c r="C257" t="s">
+        <v>21</v>
+      </c>
+      <c r="E257">
+        <v>1941000000</v>
+      </c>
+    </row>
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A258">
+        <v>2018</v>
+      </c>
+      <c r="B258">
+        <v>4</v>
+      </c>
+      <c r="C258" t="s">
+        <v>21</v>
+      </c>
+      <c r="E258">
+        <v>1891000000</v>
+      </c>
+    </row>
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A259">
+        <v>2018</v>
+      </c>
+      <c r="B259" t="s">
+        <v>8</v>
+      </c>
+      <c r="C259" t="s">
+        <v>21</v>
+      </c>
+      <c r="E259">
+        <v>7381000000</v>
+      </c>
+    </row>
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A260">
+        <v>2018</v>
+      </c>
+      <c r="B260">
+        <v>1</v>
+      </c>
+      <c r="C260" t="s">
+        <v>22</v>
+      </c>
+      <c r="E260">
+        <v>611600000</v>
+      </c>
+    </row>
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A261">
+        <v>2018</v>
+      </c>
+      <c r="B261">
+        <v>2</v>
+      </c>
+      <c r="C261" t="s">
+        <v>22</v>
+      </c>
+      <c r="E261">
+        <v>655162000</v>
+      </c>
+    </row>
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A262">
+        <v>2018</v>
+      </c>
+      <c r="B262">
+        <v>3</v>
+      </c>
+      <c r="C262" t="s">
+        <v>22</v>
+      </c>
+      <c r="E262">
+        <v>697232000</v>
+      </c>
+    </row>
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A263">
+        <v>2018</v>
+      </c>
+      <c r="B263">
+        <v>4</v>
+      </c>
+      <c r="C263" t="s">
+        <v>22</v>
+      </c>
+      <c r="E263">
+        <v>638799000</v>
+      </c>
+    </row>
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A264">
+        <v>2018</v>
+      </c>
+      <c r="B264" t="s">
+        <v>8</v>
+      </c>
+      <c r="C264" t="s">
+        <v>22</v>
+      </c>
+      <c r="E264">
+        <v>2602793000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>